<commit_message>
fix: preserve comps selection source flags
</commit_message>
<xml_diff>
--- a/public/downloads/Comps_Selection_Worksheet.xlsx
+++ b/public/downloads/Comps_Selection_Worksheet.xlsx
@@ -22,87 +22,87 @@
     <author>Author</author>
   </authors>
   <commentList>
-    <comment ref="Q4" authorId="0">
+    <comment ref="S4" authorId="0">
       <text>
         <r>
-          <t>重大基準の低スコア: 0</t>
+          <t>重大基準（データ定義）: businessModel, productMix, customerMarket, capitalIntensity / 低スコア数: 0</t>
         </r>
       </text>
     </comment>
-    <comment ref="Q5" authorId="0">
+    <comment ref="S5" authorId="0">
       <text>
         <r>
-          <t>重大基準の低スコア: 0</t>
+          <t>重大基準（データ定義）: businessModel, productMix, customerMarket, capitalIntensity / 低スコア数: 0</t>
         </r>
       </text>
     </comment>
-    <comment ref="Q6" authorId="0">
+    <comment ref="S6" authorId="0">
       <text>
         <r>
-          <t>重大基準の低スコア: 0</t>
+          <t>重大基準（データ定義）: businessModel, productMix, customerMarket, capitalIntensity / 低スコア数: 0</t>
         </r>
       </text>
     </comment>
-    <comment ref="Q7" authorId="0">
+    <comment ref="S7" authorId="0">
       <text>
         <r>
-          <t>重大基準の低スコア: 0</t>
+          <t>重大基準（データ定義）: businessModel, productMix, customerMarket, capitalIntensity / 低スコア数: 0</t>
         </r>
       </text>
     </comment>
-    <comment ref="Q8" authorId="0">
+    <comment ref="S8" authorId="0">
       <text>
         <r>
-          <t>重大基準の低スコア: 0</t>
+          <t>重大基準（データ定義）: businessModel, productMix, customerMarket, capitalIntensity / 低スコア数: 0</t>
         </r>
       </text>
     </comment>
-    <comment ref="Q9" authorId="0">
+    <comment ref="S9" authorId="0">
       <text>
         <r>
-          <t>重大基準の低スコア: 0</t>
+          <t>重大基準（データ定義）: businessModel, productMix, customerMarket, capitalIntensity / 低スコア数: 0</t>
         </r>
       </text>
     </comment>
-    <comment ref="Q10" authorId="0">
+    <comment ref="S10" authorId="0">
       <text>
         <r>
-          <t>重大基準の低スコア: 0</t>
+          <t>重大基準（データ定義）: businessModel, productMix, customerMarket, capitalIntensity / 低スコア数: 0</t>
         </r>
       </text>
     </comment>
-    <comment ref="Q11" authorId="0">
+    <comment ref="S11" authorId="0">
       <text>
         <r>
-          <t>重大基準の低スコア: 2</t>
+          <t>重大基準（データ定義）: businessModel, productMix, customerMarket, capitalIntensity / 低スコア数: 2</t>
         </r>
       </text>
     </comment>
-    <comment ref="Q12" authorId="0">
+    <comment ref="S12" authorId="0">
       <text>
         <r>
-          <t>重大基準の低スコア: 4</t>
+          <t>重大基準（データ定義）: businessModel, productMix, customerMarket, capitalIntensity / 低スコア数: 4</t>
         </r>
       </text>
     </comment>
-    <comment ref="Q13" authorId="0">
+    <comment ref="S13" authorId="0">
       <text>
         <r>
-          <t>重大基準の低スコア: 0</t>
+          <t>重大基準（データ定義）: businessModel, productMix, customerMarket, capitalIntensity / 低スコア数: 0</t>
         </r>
       </text>
     </comment>
-    <comment ref="Q14" authorId="0">
+    <comment ref="S14" authorId="0">
       <text>
         <r>
-          <t>重大基準の低スコア: 4</t>
+          <t>重大基準（データ定義）: businessModel, productMix, customerMarket, capitalIntensity / 低スコア数: 4</t>
         </r>
       </text>
     </comment>
-    <comment ref="Q15" authorId="0">
+    <comment ref="S15" authorId="0">
       <text>
         <r>
-          <t>重大基準の低スコア: 2</t>
+          <t>重大基準（データ定義）: businessModel, productMix, customerMarket, capitalIntensity / 低スコア数: 2</t>
         </r>
       </text>
     </comment>
@@ -111,7 +111,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="187">
   <si>
     <t>Comps Selection Worksheet</t>
   </si>
@@ -509,7 +509,7 @@
     <t>Selection Matrix</t>
   </si>
   <si>
-    <t>0〜3点で採点（0=不一致、3=高い一致）。重大基準の不一致はRole判断時に必ず確認します。</t>
+    <t>0〜3点で採点（0=不一致、3=高い一致）。重大基準の不一致はTask 1データのフラグを保持し、低スコアは別列で補足します。</t>
   </si>
   <si>
     <t>Role</t>
@@ -536,7 +536,13 @@
     <t>流動性</t>
   </si>
   <si>
-    <t>重大基準</t>
+    <t>重大基準の不一致</t>
+  </si>
+  <si>
+    <t>Role（source）</t>
+  </si>
+  <si>
+    <t>重大基準の低スコア</t>
   </si>
   <si>
     <t>コメント</t>
@@ -648,9 +654,6 @@
   </si>
   <si>
     <t>0が望ましい</t>
-  </si>
-  <si>
-    <t>重大基準の不一致</t>
   </si>
   <si>
     <t>Roleと根拠を確認</t>
@@ -811,7 +814,14 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="5">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFDECEC"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1175,6 +1185,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
@@ -1343,13 +1356,16 @@
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
@@ -1499,13 +1515,16 @@
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A2:C2"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:K15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
@@ -2013,25 +2032,31 @@
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A2:K2"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R15"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:T15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="15" width="13" customWidth="1"/>
-    <col min="16" max="17" width="14" customWidth="1"/>
-    <col min="18" max="18" width="58" customWidth="1"/>
+    <col min="16" max="16" width="14" customWidth="1"/>
+    <col min="17" max="17" width="18" customWidth="1"/>
+    <col min="18" max="18" width="24" customWidth="1"/>
+    <col min="19" max="19" width="18" customWidth="1"/>
+    <col min="20" max="20" width="58" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>131</v>
       </c>
@@ -2052,8 +2077,10 @@
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
-    </row>
-    <row r="2" ht="30" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S1" s="1"/>
+      <c r="T1" s="1"/>
+    </row>
+    <row r="2" ht="30" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>132</v>
       </c>
@@ -2074,8 +2101,10 @@
       <c r="P2" s="2"/>
       <c r="Q2" s="2"/>
       <c r="R2" s="2"/>
-    </row>
-    <row r="3" ht="34" customHeight="1" spans="1:18" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="S2" s="2"/>
+      <c r="T2" s="2"/>
+    </row>
+    <row r="3" ht="34" customHeight="1" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>70</v>
       </c>
@@ -2130,8 +2159,14 @@
       <c r="R3" s="4" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="4" ht="58" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S3" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="T3" s="4" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="4" ht="58" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>78</v>
       </c>
@@ -2180,14 +2215,20 @@
       <c r="P4" s="12">
         <f>SUM(D4:O4)</f>
       </c>
-      <c r="Q4" s="13">
-        <f>COUNTIF(D4:F4,"&lt;2")+COUNTIF(K4:K4,"&lt;2")</f>
+      <c r="Q4" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="R4" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="S4" s="13">
+        <f>COUNTIF(D4:D4,"&lt;2")+COUNTIF(E4:E4,"&lt;2")+COUNTIF(F4:F4,"&lt;2")+COUNTIF(K4:K4,"&lt;2")</f>
+      </c>
+      <c r="T4" s="5" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="5" ht="58" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="5" ht="58" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>84</v>
       </c>
@@ -2236,14 +2277,20 @@
       <c r="P5" s="12">
         <f>SUM(D5:O5)</f>
       </c>
-      <c r="Q5" s="13">
-        <f>COUNTIF(D5:F5,"&lt;2")+COUNTIF(K5:K5,"&lt;2")</f>
+      <c r="Q5" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="R5" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="S5" s="13">
+        <f>COUNTIF(D5:D5,"&lt;2")+COUNTIF(E5:E5,"&lt;2")+COUNTIF(F5:F5,"&lt;2")+COUNTIF(K5:K5,"&lt;2")</f>
+      </c>
+      <c r="T5" s="5" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="6" ht="58" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="6" ht="58" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>88</v>
       </c>
@@ -2292,14 +2339,20 @@
       <c r="P6" s="12">
         <f>SUM(D6:O6)</f>
       </c>
-      <c r="Q6" s="13">
-        <f>COUNTIF(D6:F6,"&lt;2")+COUNTIF(K6:K6,"&lt;2")</f>
+      <c r="Q6" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="R6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="S6" s="13">
+        <f>COUNTIF(D6:D6,"&lt;2")+COUNTIF(E6:E6,"&lt;2")+COUNTIF(F6:F6,"&lt;2")+COUNTIF(K6:K6,"&lt;2")</f>
+      </c>
+      <c r="T6" s="5" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="7" ht="58" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="7" ht="58" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>92</v>
       </c>
@@ -2348,14 +2401,20 @@
       <c r="P7" s="12">
         <f>SUM(D7:O7)</f>
       </c>
-      <c r="Q7" s="13">
-        <f>COUNTIF(D7:F7,"&lt;2")+COUNTIF(K7:K7,"&lt;2")</f>
+      <c r="Q7" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="R7" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="S7" s="13">
+        <f>COUNTIF(D7:D7,"&lt;2")+COUNTIF(E7:E7,"&lt;2")+COUNTIF(F7:F7,"&lt;2")+COUNTIF(K7:K7,"&lt;2")</f>
+      </c>
+      <c r="T7" s="5" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="8" ht="58" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="8" ht="58" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>96</v>
       </c>
@@ -2404,14 +2463,20 @@
       <c r="P8" s="12">
         <f>SUM(D8:O8)</f>
       </c>
-      <c r="Q8" s="13">
-        <f>COUNTIF(D8:F8,"&lt;2")+COUNTIF(K8:K8,"&lt;2")</f>
+      <c r="Q8" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="R8" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="S8" s="13">
+        <f>COUNTIF(D8:D8,"&lt;2")+COUNTIF(E8:E8,"&lt;2")+COUNTIF(F8:F8,"&lt;2")+COUNTIF(K8:K8,"&lt;2")</f>
+      </c>
+      <c r="T8" s="5" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="9" ht="58" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="9" ht="58" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>100</v>
       </c>
@@ -2460,14 +2525,20 @@
       <c r="P9" s="12">
         <f>SUM(D9:O9)</f>
       </c>
-      <c r="Q9" s="13">
-        <f>COUNTIF(D9:F9,"&lt;2")+COUNTIF(K9:K9,"&lt;2")</f>
+      <c r="Q9" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="R9" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="S9" s="13">
+        <f>COUNTIF(D9:D9,"&lt;2")+COUNTIF(E9:E9,"&lt;2")+COUNTIF(F9:F9,"&lt;2")+COUNTIF(K9:K9,"&lt;2")</f>
+      </c>
+      <c r="T9" s="5" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="10" ht="58" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="10" ht="58" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>104</v>
       </c>
@@ -2516,14 +2587,20 @@
       <c r="P10" s="12">
         <f>SUM(D10:O10)</f>
       </c>
-      <c r="Q10" s="13">
-        <f>COUNTIF(D10:F10,"&lt;2")+COUNTIF(K10:K10,"&lt;2")</f>
+      <c r="Q10" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="R10" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="S10" s="13">
+        <f>COUNTIF(D10:D10,"&lt;2")+COUNTIF(E10:E10,"&lt;2")+COUNTIF(F10:F10,"&lt;2")+COUNTIF(K10:K10,"&lt;2")</f>
+      </c>
+      <c r="T10" s="5" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="11" ht="58" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="11" ht="58" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>109</v>
       </c>
@@ -2572,14 +2649,20 @@
       <c r="P11" s="12">
         <f>SUM(D11:O11)</f>
       </c>
-      <c r="Q11" s="13">
-        <f>COUNTIF(D11:F11,"&lt;2")+COUNTIF(K11:K11,"&lt;2")</f>
+      <c r="Q11" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="R11" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="S11" s="13">
+        <f>COUNTIF(D11:D11,"&lt;2")+COUNTIF(E11:E11,"&lt;2")+COUNTIF(F11:F11,"&lt;2")+COUNTIF(K11:K11,"&lt;2")</f>
+      </c>
+      <c r="T11" s="5" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="12" ht="58" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="12" ht="58" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>113</v>
       </c>
@@ -2628,14 +2711,20 @@
       <c r="P12" s="12">
         <f>SUM(D12:O12)</f>
       </c>
-      <c r="Q12" s="13">
-        <f>COUNTIF(D12:F12,"&lt;2")+COUNTIF(K12:K12,"&lt;2")</f>
+      <c r="Q12" s="5" t="b">
+        <v>1</v>
       </c>
       <c r="R12" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="S12" s="13">
+        <f>COUNTIF(D12:D12,"&lt;2")+COUNTIF(E12:E12,"&lt;2")+COUNTIF(F12:F12,"&lt;2")+COUNTIF(K12:K12,"&lt;2")</f>
+      </c>
+      <c r="T12" s="5" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="13" ht="58" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="13" ht="58" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>117</v>
       </c>
@@ -2684,14 +2773,20 @@
       <c r="P13" s="12">
         <f>SUM(D13:O13)</f>
       </c>
-      <c r="Q13" s="13">
-        <f>COUNTIF(D13:F13,"&lt;2")+COUNTIF(K13:K13,"&lt;2")</f>
+      <c r="Q13" s="5" t="b">
+        <v>1</v>
       </c>
       <c r="R13" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="S13" s="13">
+        <f>COUNTIF(D13:D13,"&lt;2")+COUNTIF(E13:E13,"&lt;2")+COUNTIF(F13:F13,"&lt;2")+COUNTIF(K13:K13,"&lt;2")</f>
+      </c>
+      <c r="T13" s="5" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="14" ht="58" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="14" ht="58" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>122</v>
       </c>
@@ -2740,14 +2835,20 @@
       <c r="P14" s="12">
         <f>SUM(D14:O14)</f>
       </c>
-      <c r="Q14" s="13">
-        <f>COUNTIF(D14:F14,"&lt;2")+COUNTIF(K14:K14,"&lt;2")</f>
+      <c r="Q14" s="5" t="b">
+        <v>1</v>
       </c>
       <c r="R14" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="S14" s="13">
+        <f>COUNTIF(D14:D14,"&lt;2")+COUNTIF(E14:E14,"&lt;2")+COUNTIF(F14:F14,"&lt;2")+COUNTIF(K14:K14,"&lt;2")</f>
+      </c>
+      <c r="T14" s="5" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="15" ht="58" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="15" ht="58" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>127</v>
       </c>
@@ -2796,18 +2897,24 @@
       <c r="P15" s="12">
         <f>SUM(D15:O15)</f>
       </c>
-      <c r="Q15" s="13">
-        <f>COUNTIF(D15:F15,"&lt;2")+COUNTIF(K15:K15,"&lt;2")</f>
+      <c r="Q15" s="5" t="b">
+        <v>1</v>
       </c>
       <c r="R15" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="S15" s="13">
+        <f>COUNTIF(D15:D15,"&lt;2")+COUNTIF(E15:E15,"&lt;2")+COUNTIF(F15:F15,"&lt;2")+COUNTIF(K15:K15,"&lt;2")</f>
+      </c>
+      <c r="T15" s="5" t="s">
         <v>130</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:R15"/>
+  <autoFilter ref="A3:T15"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:R1"/>
-    <mergeCell ref="A2:R2"/>
+    <mergeCell ref="A1:T1"/>
+    <mergeCell ref="A2:T2"/>
   </mergeCells>
   <conditionalFormatting sqref="D4:O15">
     <cfRule type="colorScale" priority="1">
@@ -2822,18 +2929,26 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q4:Q15">
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
+      <formula>TRUE</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S4:S15">
+    <cfRule type="cellIs" dxfId="1" priority="3" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:F16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
@@ -2847,7 +2962,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2857,7 +2972,7 @@
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2876,13 +2991,13 @@
         <v>133</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="5" ht="70" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -2899,10 +3014,10 @@
         <v>83</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="6" ht="70" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -2919,10 +3034,10 @@
         <v>87</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="7" ht="70" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -2939,10 +3054,10 @@
         <v>91</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="8" ht="70" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -2959,10 +3074,10 @@
         <v>95</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="9" ht="70" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -2979,10 +3094,10 @@
         <v>99</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="10" ht="70" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -2999,10 +3114,10 @@
         <v>103</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="11" ht="70" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -3019,10 +3134,10 @@
         <v>108</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="12" ht="70" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -3039,10 +3154,10 @@
         <v>112</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="13" ht="70" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -3059,10 +3174,10 @@
         <v>116</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="14" ht="70" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -3079,10 +3194,10 @@
         <v>121</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="15" ht="70" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -3099,10 +3214,10 @@
         <v>126</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="16" ht="70" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -3119,10 +3234,10 @@
         <v>130</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
   </sheetData>
@@ -3139,13 +3254,16 @@
       <formula1>"core_peer,secondary_peer,aspirational_peer,negative_peer,excluded_close_peer,not_clean_comp"</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
@@ -3157,7 +3275,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3165,7 +3283,7 @@
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3173,30 +3291,30 @@
     </row>
     <row r="4" ht="34" customHeight="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="5" ht="50" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B5" s="5">
         <f>COUNTIF('Peer Roles'!$C$5:$C$16,"core_peer")</f>
       </c>
       <c r="C5" s="5" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="6" ht="50" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -3207,66 +3325,66 @@
         <f>TEXTJOIN(", ",TRUE,IF('Peer Roles'!$C$5:$C$16="core_peer",'Peer Roles'!$B$5:$B$16,""))</f>
       </c>
       <c r="C6" s="5" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="7" ht="50" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B7" s="5">
         <f>TEXTJOIN(", ",TRUE,IF('Peer Roles'!$C$5:$C$16="secondary_peer",'Peer Roles'!$B$5:$B$16,""))</f>
       </c>
       <c r="C7" s="5" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="8" ht="50" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B8" s="5">
         <f>TEXTJOIN(", ",TRUE,IF(('Peer Roles'!$C$5:$C$16="excluded_close_peer")+('Peer Roles'!$C$5:$C$16="not_clean_comp"),'Peer Roles'!$B$5:$B$16,""))</f>
       </c>
       <c r="C8" s="5" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="9" ht="50" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B9" s="5">
         <f>COUNTIF('Peer Roles'!$F$5:$F$16,"未確認")</f>
       </c>
       <c r="C9" s="5" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="10" ht="50" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
   </sheetData>
@@ -3275,13 +3393,16 @@
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
@@ -3292,93 +3413,93 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B4" s="5">
         <f>COUNTBLANK('Peer Roles'!$C$5:$C$16)</f>
       </c>
       <c r="C4" s="5" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B5" s="5">
         <f>COUNTIF('Peer Roles'!$F$5:$F$16,"未確認")</f>
       </c>
       <c r="C5" s="5" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>179</v>
+        <v>141</v>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('Selection Matrix'!$Q$4:$Q$15,"&gt;0")</f>
+        <f>COUNTIF('Selection Matrix'!$Q$4:$Q$15,TRUE)</f>
       </c>
       <c r="C6" s="5" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B7" s="5">
         <f>COUNTIF('Peer Roles'!$C$5:$C$16,"core_peer")</f>
       </c>
       <c r="C7" s="5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B8" s="5">
         <f>COUNTA('Peer Roles'!$A$5:$A$16)</f>
       </c>
       <c r="C8" s="5" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
   </sheetData>
@@ -3388,21 +3509,21 @@
     <mergeCell ref="A2:C2"/>
   </mergeCells>
   <conditionalFormatting sqref="B4:B4">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B5:B5">
-    <cfRule type="cellIs" dxfId="2" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="3" priority="2" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:B6">
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="4" priority="3" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: strengthen comps selection controls
</commit_message>
<xml_diff>
--- a/public/downloads/Comps_Selection_Worksheet.xlsx
+++ b/public/downloads/Comps_Selection_Worksheet.xlsx
@@ -22,84 +22,84 @@
     <author>Author</author>
   </authors>
   <commentList>
-    <comment ref="S4" authorId="0">
+    <comment ref="U4" authorId="0">
       <text>
         <r>
           <t>重大基準（データ定義）: businessModel, productMix, customerMarket, capitalIntensity / 低スコア数: 0</t>
         </r>
       </text>
     </comment>
-    <comment ref="S5" authorId="0">
+    <comment ref="U5" authorId="0">
       <text>
         <r>
           <t>重大基準（データ定義）: businessModel, productMix, customerMarket, capitalIntensity / 低スコア数: 0</t>
         </r>
       </text>
     </comment>
-    <comment ref="S6" authorId="0">
+    <comment ref="U6" authorId="0">
       <text>
         <r>
           <t>重大基準（データ定義）: businessModel, productMix, customerMarket, capitalIntensity / 低スコア数: 0</t>
         </r>
       </text>
     </comment>
-    <comment ref="S7" authorId="0">
+    <comment ref="U7" authorId="0">
       <text>
         <r>
           <t>重大基準（データ定義）: businessModel, productMix, customerMarket, capitalIntensity / 低スコア数: 0</t>
         </r>
       </text>
     </comment>
-    <comment ref="S8" authorId="0">
+    <comment ref="U8" authorId="0">
       <text>
         <r>
           <t>重大基準（データ定義）: businessModel, productMix, customerMarket, capitalIntensity / 低スコア数: 0</t>
         </r>
       </text>
     </comment>
-    <comment ref="S9" authorId="0">
+    <comment ref="U9" authorId="0">
       <text>
         <r>
           <t>重大基準（データ定義）: businessModel, productMix, customerMarket, capitalIntensity / 低スコア数: 0</t>
         </r>
       </text>
     </comment>
-    <comment ref="S10" authorId="0">
+    <comment ref="U10" authorId="0">
       <text>
         <r>
           <t>重大基準（データ定義）: businessModel, productMix, customerMarket, capitalIntensity / 低スコア数: 0</t>
         </r>
       </text>
     </comment>
-    <comment ref="S11" authorId="0">
+    <comment ref="U11" authorId="0">
       <text>
         <r>
           <t>重大基準（データ定義）: businessModel, productMix, customerMarket, capitalIntensity / 低スコア数: 2</t>
         </r>
       </text>
     </comment>
-    <comment ref="S12" authorId="0">
+    <comment ref="U12" authorId="0">
       <text>
         <r>
           <t>重大基準（データ定義）: businessModel, productMix, customerMarket, capitalIntensity / 低スコア数: 4</t>
         </r>
       </text>
     </comment>
-    <comment ref="S13" authorId="0">
+    <comment ref="U13" authorId="0">
       <text>
         <r>
           <t>重大基準（データ定義）: businessModel, productMix, customerMarket, capitalIntensity / 低スコア数: 0</t>
         </r>
       </text>
     </comment>
-    <comment ref="S14" authorId="0">
+    <comment ref="U14" authorId="0">
       <text>
         <r>
           <t>重大基準（データ定義）: businessModel, productMix, customerMarket, capitalIntensity / 低スコア数: 4</t>
         </r>
       </text>
     </comment>
-    <comment ref="S15" authorId="0">
+    <comment ref="U15" authorId="0">
       <text>
         <r>
           <t>重大基準（データ定義）: businessModel, productMix, customerMarket, capitalIntensity / 低スコア数: 2</t>
@@ -111,7 +111,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="191">
   <si>
     <t>Comps Selection Worksheet</t>
   </si>
@@ -509,7 +509,7 @@
     <t>Selection Matrix</t>
   </si>
   <si>
-    <t>0〜3点で採点（0=不一致、3=高い一致）。重大基準の不一致はTask 1データのフラグを保持し、低スコアは別列で補足します。</t>
+    <t>0〜3点で採点。重大基準の不一致、データ欠損、Core適格性ブロックを分けて記録します。</t>
   </si>
   <si>
     <t>Role</t>
@@ -539,7 +539,13 @@
     <t>重大基準の不一致</t>
   </si>
   <si>
-    <t>Role（source）</t>
+    <t>データ欠損</t>
+  </si>
+  <si>
+    <t>Core適格性ブロック</t>
+  </si>
+  <si>
+    <t>Role（Source）</t>
   </si>
   <si>
     <t>重大基準の低スコア</t>
@@ -548,10 +554,16 @@
     <t>コメント</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
+    <t>margin, liquidity</t>
+  </si>
+  <si>
     <t>Peer Roles</t>
   </si>
   <si>
-    <t>Roleを分類し、採用・除外の根拠と追加調査事項を残します。Role列はプルダウンから選択します。</t>
+    <t>Roleと根拠に加え、重大不一致、データ欠損、Core適格性ブロックを独立して確認します。</t>
   </si>
   <si>
     <t>採用・除外の根拠</t>
@@ -569,10 +581,10 @@
     <t>利用可</t>
   </si>
   <si>
-    <t>EBITDAマージンの確認</t>
-  </si>
-  <si>
-    <t>未確認</t>
+    <t>margin, liquidityの確認</t>
+  </si>
+  <si>
+    <t>一部未確認</t>
   </si>
   <si>
     <t>Review Memo</t>
@@ -599,9 +611,6 @@
     <t>中心レンジとして十分な数か</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>名称とRoleを確認</t>
   </si>
   <si>
@@ -650,19 +659,22 @@
     <t>0であること</t>
   </si>
   <si>
-    <t>データ未確認</t>
-  </si>
-  <si>
-    <t>0が望ましい</t>
-  </si>
-  <si>
-    <t>Roleと根拠を確認</t>
+    <t>理由未入力</t>
+  </si>
+  <si>
+    <t>ID重複</t>
+  </si>
+  <si>
+    <t>Core＋重大不一致</t>
+  </si>
+  <si>
+    <t>Core＋データ欠損</t>
   </si>
   <si>
     <t>5〜8社を目安</t>
   </si>
   <si>
-    <t>候補数</t>
+    <t>候補社数</t>
   </si>
   <si>
     <t>12社であること</t>
@@ -814,7 +826,28 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
+  <dxfs count="8">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFDECEC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFDECEC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFDECEC"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -2042,7 +2075,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:T15"/>
+  <dimension ref="A1:V15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -2051,12 +2084,14 @@
     <col min="4" max="15" width="13" customWidth="1"/>
     <col min="16" max="16" width="14" customWidth="1"/>
     <col min="17" max="17" width="18" customWidth="1"/>
-    <col min="18" max="18" width="24" customWidth="1"/>
-    <col min="19" max="19" width="18" customWidth="1"/>
-    <col min="20" max="20" width="58" customWidth="1"/>
+    <col min="18" max="18" width="22" customWidth="1"/>
+    <col min="19" max="19" width="20" customWidth="1"/>
+    <col min="20" max="20" width="24" customWidth="1"/>
+    <col min="21" max="21" width="18" customWidth="1"/>
+    <col min="22" max="22" width="58" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="1" ht="28" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>131</v>
       </c>
@@ -2079,8 +2114,10 @@
       <c r="R1" s="1"/>
       <c r="S1" s="1"/>
       <c r="T1" s="1"/>
-    </row>
-    <row r="2" ht="30" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U1" s="1"/>
+      <c r="V1" s="1"/>
+    </row>
+    <row r="2" ht="30" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>132</v>
       </c>
@@ -2103,8 +2140,10 @@
       <c r="R2" s="2"/>
       <c r="S2" s="2"/>
       <c r="T2" s="2"/>
-    </row>
-    <row r="3" ht="34" customHeight="1" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="U2" s="2"/>
+      <c r="V2" s="2"/>
+    </row>
+    <row r="3" ht="34" customHeight="1" spans="1:22" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>70</v>
       </c>
@@ -2165,8 +2204,14 @@
       <c r="T3" s="4" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="4" ht="58" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U3" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="V3" s="4" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="4" ht="58" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>78</v>
       </c>
@@ -2219,16 +2264,22 @@
         <v>0</v>
       </c>
       <c r="R4" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="S4" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="T4" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="S4" s="13">
+      <c r="U4" s="13">
         <f>COUNTIF(D4:D4,"&lt;2")+COUNTIF(E4:E4,"&lt;2")+COUNTIF(F4:F4,"&lt;2")+COUNTIF(K4:K4,"&lt;2")</f>
       </c>
-      <c r="T4" s="5" t="s">
+      <c r="V4" s="5" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="5" ht="58" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="5" ht="58" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>84</v>
       </c>
@@ -2281,16 +2332,22 @@
         <v>0</v>
       </c>
       <c r="R5" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="S5" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="T5" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="S5" s="13">
+      <c r="U5" s="13">
         <f>COUNTIF(D5:D5,"&lt;2")+COUNTIF(E5:E5,"&lt;2")+COUNTIF(F5:F5,"&lt;2")+COUNTIF(K5:K5,"&lt;2")</f>
       </c>
-      <c r="T5" s="5" t="s">
+      <c r="V5" s="5" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="6" ht="58" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="6" ht="58" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>88</v>
       </c>
@@ -2343,16 +2400,22 @@
         <v>0</v>
       </c>
       <c r="R6" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="S6" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="T6" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="S6" s="13">
+      <c r="U6" s="13">
         <f>COUNTIF(D6:D6,"&lt;2")+COUNTIF(E6:E6,"&lt;2")+COUNTIF(F6:F6,"&lt;2")+COUNTIF(K6:K6,"&lt;2")</f>
       </c>
-      <c r="T6" s="5" t="s">
+      <c r="V6" s="5" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="7" ht="58" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="7" ht="58" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>92</v>
       </c>
@@ -2405,16 +2468,22 @@
         <v>0</v>
       </c>
       <c r="R7" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="S7" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="T7" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="S7" s="13">
+      <c r="U7" s="13">
         <f>COUNTIF(D7:D7,"&lt;2")+COUNTIF(E7:E7,"&lt;2")+COUNTIF(F7:F7,"&lt;2")+COUNTIF(K7:K7,"&lt;2")</f>
       </c>
-      <c r="T7" s="5" t="s">
+      <c r="V7" s="5" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="8" ht="58" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="8" ht="58" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>96</v>
       </c>
@@ -2467,16 +2536,22 @@
         <v>0</v>
       </c>
       <c r="R8" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="S8" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="T8" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="S8" s="13">
+      <c r="U8" s="13">
         <f>COUNTIF(D8:D8,"&lt;2")+COUNTIF(E8:E8,"&lt;2")+COUNTIF(F8:F8,"&lt;2")+COUNTIF(K8:K8,"&lt;2")</f>
       </c>
-      <c r="T8" s="5" t="s">
+      <c r="V8" s="5" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="9" ht="58" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="9" ht="58" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>100</v>
       </c>
@@ -2529,16 +2604,22 @@
         <v>0</v>
       </c>
       <c r="R9" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="S9" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="T9" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="S9" s="13">
+      <c r="U9" s="13">
         <f>COUNTIF(D9:D9,"&lt;2")+COUNTIF(E9:E9,"&lt;2")+COUNTIF(F9:F9,"&lt;2")+COUNTIF(K9:K9,"&lt;2")</f>
       </c>
-      <c r="T9" s="5" t="s">
+      <c r="V9" s="5" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="10" ht="58" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="10" ht="58" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>104</v>
       </c>
@@ -2591,16 +2672,22 @@
         <v>0</v>
       </c>
       <c r="R10" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="S10" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="T10" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="S10" s="13">
+      <c r="U10" s="13">
         <f>COUNTIF(D10:D10,"&lt;2")+COUNTIF(E10:E10,"&lt;2")+COUNTIF(F10:F10,"&lt;2")+COUNTIF(K10:K10,"&lt;2")</f>
       </c>
-      <c r="T10" s="5" t="s">
+      <c r="V10" s="5" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="11" ht="58" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="11" ht="58" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>109</v>
       </c>
@@ -2650,19 +2737,25 @@
         <f>SUM(D11:O11)</f>
       </c>
       <c r="Q11" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R11" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="S11" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="T11" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="S11" s="13">
+      <c r="U11" s="13">
         <f>COUNTIF(D11:D11,"&lt;2")+COUNTIF(E11:E11,"&lt;2")+COUNTIF(F11:F11,"&lt;2")+COUNTIF(K11:K11,"&lt;2")</f>
       </c>
-      <c r="T11" s="5" t="s">
+      <c r="V11" s="5" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="12" ht="58" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="12" ht="58" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>113</v>
       </c>
@@ -2715,16 +2808,22 @@
         <v>1</v>
       </c>
       <c r="R12" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="S12" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="T12" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="S12" s="13">
+      <c r="U12" s="13">
         <f>COUNTIF(D12:D12,"&lt;2")+COUNTIF(E12:E12,"&lt;2")+COUNTIF(F12:F12,"&lt;2")+COUNTIF(K12:K12,"&lt;2")</f>
       </c>
-      <c r="T12" s="5" t="s">
+      <c r="V12" s="5" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="13" ht="58" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="13" ht="58" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>117</v>
       </c>
@@ -2752,8 +2851,8 @@
       <c r="I13" s="11">
         <v>3</v>
       </c>
-      <c r="J13" s="11">
-        <v>0</v>
+      <c r="J13" s="11" t="s">
+        <v>120</v>
       </c>
       <c r="K13" s="11">
         <v>3</v>
@@ -2767,26 +2866,32 @@
       <c r="N13" s="11">
         <v>3</v>
       </c>
-      <c r="O13" s="11">
-        <v>0</v>
+      <c r="O13" s="11" t="s">
+        <v>120</v>
       </c>
       <c r="P13" s="12">
         <f>SUM(D13:O13)</f>
       </c>
       <c r="Q13" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="R13" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="S13" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="R13" s="5" t="s">
+      <c r="T13" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="S13" s="13">
+      <c r="U13" s="13">
         <f>COUNTIF(D13:D13,"&lt;2")+COUNTIF(E13:E13,"&lt;2")+COUNTIF(F13:F13,"&lt;2")+COUNTIF(K13:K13,"&lt;2")</f>
       </c>
-      <c r="T13" s="5" t="s">
+      <c r="V13" s="5" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="14" ht="58" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="14" ht="58" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>122</v>
       </c>
@@ -2839,16 +2944,22 @@
         <v>1</v>
       </c>
       <c r="R14" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="S14" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="T14" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="S14" s="13">
+      <c r="U14" s="13">
         <f>COUNTIF(D14:D14,"&lt;2")+COUNTIF(E14:E14,"&lt;2")+COUNTIF(F14:F14,"&lt;2")+COUNTIF(K14:K14,"&lt;2")</f>
       </c>
-      <c r="T14" s="5" t="s">
+      <c r="V14" s="5" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="15" ht="58" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="15" ht="58" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>127</v>
       </c>
@@ -2901,20 +3012,26 @@
         <v>1</v>
       </c>
       <c r="R15" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="S15" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="T15" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="S15" s="13">
+      <c r="U15" s="13">
         <f>COUNTIF(D15:D15,"&lt;2")+COUNTIF(E15:E15,"&lt;2")+COUNTIF(F15:F15,"&lt;2")+COUNTIF(K15:K15,"&lt;2")</f>
       </c>
-      <c r="T15" s="5" t="s">
+      <c r="V15" s="5" t="s">
         <v>130</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:T15"/>
+  <autoFilter ref="A3:V15"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:T1"/>
-    <mergeCell ref="A2:T2"/>
+    <mergeCell ref="A1:V1"/>
+    <mergeCell ref="A2:V2"/>
   </mergeCells>
   <conditionalFormatting sqref="D4:O15">
     <cfRule type="colorScale" priority="1">
@@ -2949,7 +3066,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -2958,29 +3075,38 @@
     <col min="4" max="4" width="58" customWidth="1"/>
     <col min="5" max="5" width="32" customWidth="1"/>
     <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="7" max="7" width="18" customWidth="1"/>
+    <col min="8" max="8" width="22" customWidth="1"/>
+    <col min="9" max="9" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
-    </row>
-    <row r="2" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+    </row>
+    <row r="2" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
-    </row>
-    <row r="4" ht="34" customHeight="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+    </row>
+    <row r="4" ht="34" customHeight="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>70</v>
       </c>
@@ -2991,16 +3117,25 @@
         <v>133</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="5" ht="70" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+        <v>153</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="5" ht="70" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>78</v>
       </c>
@@ -3014,13 +3149,22 @@
         <v>83</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="6" ht="70" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+        <v>155</v>
+      </c>
+      <c r="G5" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="I5" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" ht="70" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>84</v>
       </c>
@@ -3034,13 +3178,22 @@
         <v>87</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="7" ht="70" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+        <v>155</v>
+      </c>
+      <c r="G6" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="I6" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" ht="70" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>88</v>
       </c>
@@ -3054,13 +3207,22 @@
         <v>91</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="8" ht="70" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+        <v>155</v>
+      </c>
+      <c r="G7" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="I7" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" ht="70" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>92</v>
       </c>
@@ -3074,13 +3236,22 @@
         <v>95</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="9" ht="70" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+        <v>155</v>
+      </c>
+      <c r="G8" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="I8" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" ht="70" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>96</v>
       </c>
@@ -3094,13 +3265,22 @@
         <v>99</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="10" ht="70" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+        <v>155</v>
+      </c>
+      <c r="G9" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="I9" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" ht="70" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>100</v>
       </c>
@@ -3114,13 +3294,22 @@
         <v>103</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="11" ht="70" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+        <v>155</v>
+      </c>
+      <c r="G10" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="I10" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" ht="70" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>104</v>
       </c>
@@ -3134,13 +3323,22 @@
         <v>108</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="12" ht="70" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+        <v>155</v>
+      </c>
+      <c r="G11" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="I11" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" ht="70" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>109</v>
       </c>
@@ -3154,13 +3352,22 @@
         <v>112</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="13" ht="70" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+        <v>155</v>
+      </c>
+      <c r="G12" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="I12" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" ht="70" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>113</v>
       </c>
@@ -3174,13 +3381,22 @@
         <v>116</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="14" ht="70" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+        <v>155</v>
+      </c>
+      <c r="G13" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="I13" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" ht="70" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>117</v>
       </c>
@@ -3194,13 +3410,22 @@
         <v>121</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="15" ht="70" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+        <v>157</v>
+      </c>
+      <c r="G14" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="H14" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="I14" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" ht="70" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>122</v>
       </c>
@@ -3214,13 +3439,22 @@
         <v>126</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="16" ht="70" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+        <v>155</v>
+      </c>
+      <c r="G15" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="H15" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="I15" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" ht="70" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>127</v>
       </c>
@@ -3234,17 +3468,26 @@
         <v>130</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>151</v>
+        <v>155</v>
+      </c>
+      <c r="G16" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="H16" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="I16" s="5" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:F16"/>
+  <autoFilter ref="A4:I16"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" showErrorMessage="1" errorStyle="stop" errorTitle="Roleを選択してください" error="プルダウンのRoleから選択してください。" sqref="C10:C16">
@@ -3275,7 +3518,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3283,7 +3526,7 @@
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3291,30 +3534,30 @@
     </row>
     <row r="4" ht="34" customHeight="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
     </row>
     <row r="5" ht="50" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="B5" s="5">
         <f>COUNTIF('Peer Roles'!$C$5:$C$16,"core_peer")</f>
       </c>
       <c r="C5" s="5" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>162</v>
+        <v>147</v>
       </c>
     </row>
     <row r="6" ht="50" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -3325,66 +3568,66 @@
         <f>TEXTJOIN(", ",TRUE,IF('Peer Roles'!$C$5:$C$16="core_peer",'Peer Roles'!$B$5:$B$16,""))</f>
       </c>
       <c r="C6" s="5" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>162</v>
+        <v>147</v>
       </c>
     </row>
     <row r="7" ht="50" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="B7" s="5">
         <f>TEXTJOIN(", ",TRUE,IF('Peer Roles'!$C$5:$C$16="secondary_peer",'Peer Roles'!$B$5:$B$16,""))</f>
       </c>
       <c r="C7" s="5" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>162</v>
+        <v>147</v>
       </c>
     </row>
     <row r="8" ht="50" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="B8" s="5">
         <f>TEXTJOIN(", ",TRUE,IF(('Peer Roles'!$C$5:$C$16="excluded_close_peer")+('Peer Roles'!$C$5:$C$16="not_clean_comp"),'Peer Roles'!$B$5:$B$16,""))</f>
       </c>
       <c r="C8" s="5" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>162</v>
+        <v>147</v>
       </c>
     </row>
     <row r="9" ht="50" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="B9" s="5">
         <f>COUNTIF('Peer Roles'!$F$5:$F$16,"未確認")</f>
       </c>
       <c r="C9" s="5" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>162</v>
+        <v>147</v>
       </c>
     </row>
     <row r="10" ht="50" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>162</v>
+        <v>147</v>
       </c>
     </row>
   </sheetData>
@@ -3403,7 +3646,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -3413,57 +3656,57 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="B4" s="5">
         <f>COUNTBLANK('Peer Roles'!$C$5:$C$16)</f>
       </c>
       <c r="C4" s="5" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="B5" s="5">
-        <f>COUNTIF('Peer Roles'!$F$5:$F$16,"未確認")</f>
+        <f>COUNTBLANK('Peer Roles'!$D$5:$D$16)</f>
       </c>
       <c r="C5" s="5" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>141</v>
+        <v>183</v>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('Selection Matrix'!$Q$4:$Q$15,TRUE)</f>
+        <f>SUMPRODUCT((COUNTIF('Peer Roles'!$A$5:$A$16,'Peer Roles'!$A$5:$A$16)&gt;1)*1)</f>
       </c>
       <c r="C6" s="5" t="s">
         <v>181</v>
@@ -3471,39 +3714,72 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>160</v>
+        <v>184</v>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('Peer Roles'!$C$5:$C$16,"core_peer")</f>
+        <f>COUNTIFS('Peer Roles'!$C$5:$C$16,"core_peer",'Peer Roles'!$G$5:$G$16,TRUE)</f>
       </c>
       <c r="C7" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B8" s="5">
-        <f>COUNTA('Peer Roles'!$A$5:$A$16)</f>
+        <f>COUNTIFS('Peer Roles'!$C$5:$C$16,"core_peer",'Peer Roles'!$H$5:$H$16,"?*")</f>
       </c>
       <c r="C8" s="5" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>185</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>150</v>
+        <v>143</v>
+      </c>
+      <c r="B9" s="5">
+        <f>COUNTIFS('Peer Roles'!$C$5:$C$16,"core_peer",'Peer Roles'!$I$5:$I$16,TRUE)</f>
       </c>
       <c r="C9" s="5" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="B10" s="5">
+        <f>COUNTIF('Peer Roles'!$C$5:$C$16,"core_peer")</f>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>186</v>
       </c>
     </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="B11" s="5">
+        <f>COUNTA('Peer Roles'!$A$5:$A$16)</f>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>190</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:C9"/>
+  <autoFilter ref="A3:C12"/>
   <mergeCells count="2">
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A2:C2"/>
@@ -3523,6 +3799,21 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="B7:B7">
+    <cfRule type="cellIs" dxfId="5" priority="7" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B8:B8">
+    <cfRule type="cellIs" dxfId="6" priority="8" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B9:B9">
+    <cfRule type="cellIs" dxfId="7" priority="9" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>